<commit_message>
docs+feat: odluke #10 i #11 u planu, dodatne_kategorije u Excel pipelineu
- PLAN §4.3: više kategorija (M2M + primarna, limit 3, podjela odgovornosti
  primarna/sve, pravilo usporedbe); §A: analitika (first-party, agregatno, bez PII,
  events+daily_stats, katalog eventa, POST /api/events); §M prerađen — ODOBREN:
  freemium granica M.1, Founding partner (12 mj), Statistika profila kao premium,
  Izdvojeno samo na općem pregledu, karta trajno organska; §3 modeli + faze dopunjene
- STANJE.md: log sesije + ZADACI A/B/C za sljedeću kodnu sesiju (Opus)
- Excel: stupac dodatne_kategorije (max 2, samo ';' separator — imena kategorija
  sadrže zareze) + upute + primjeri; import validira i piše categories=[primarna,...]
- Vendor.categories (opcionalno) — UI ga još ne čita (Zadatak A)
</commit_message>
<xml_diff>
--- a/data/vendors-template.xlsx
+++ b/data/vendors-template.xlsx
@@ -199,110 +199,115 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
+        <t>Najviše 2 dodatne kategorije iz šifrarnika, odvojene točka-zarezom (npr. DJ; Catering). NE ponavljati primarnu. Više od 3 ukupno: zahtjev adminu (nakon claima).</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
         <t>Odaberi iz padajućeg izbornika</t>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>SJEDIŠTE — jedan grad. Ako ih pružatelj navodi više, upiši glavni/prvi, ostale u pokrivanje_napomena. Prazno = poznata samo regija (bez pina na karti). OBAVEZNO za sale/konobe/kuće za proslavu.</t>
       </text>
     </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Google Maps → desni klik na lokaciju → klik na koordinate (kopira "43.5081, 16.4402") → zalijepi ovdje. Prazno = geokodira se iz grada (Faza 1). OBAVEZNO za sale/konobe/kuće za proslavu. Nikad ne izmišljaj koordinatu!</t>
       </text>
     </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Gdje pružatelj RADI (uz svoju regiju). Više regija odvoji točka-zarezom: Dalmacija; Kvarner. Za cijelu državu upiši: cijela Hrvatska. Prazno = radi samo u svojoj regiji.</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Slobodni tekst o pokrivanju, npr. 'radi u Splitu, Zadru i Šibeniku' ili 'po dogovoru i BiH'. Prikazuje se na profilu.</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
+    <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>od (paušal) = jedna cijena 'od X €'; po osobi (raspon) = X–Y €/os. (sale, catering)</t>
       </text>
     </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
+    <comment ref="J1" authorId="0" shapeId="0">
       <text>
         <t>Samo broj u €, bez oznake valute</t>
       </text>
     </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
+    <comment ref="K1" authorId="0" shapeId="0">
       <text>
         <t>Samo za 'po osobi (raspon)'</t>
       </text>
     </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
+    <comment ref="L1" authorId="0" shapeId="0">
       <text>
         <t>0–5, npr. 4.8 — prenesena ocjena (Google i sl.). Ostavi prazno ako nema.</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>OBAVEZNO ako je ocjena upisana, npr. 'Google recenzije'</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>DA = kontaktirali smo ih i potvrdili podatke</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>Zasad NE za sve — DA tek kad pružatelj dobije CRM</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>Tagovi odvojeni zarezom, npr: uz more, terasa</t>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
+    <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <t>Što pružatelj kaže o sebi (2–4 rečenice). Prazno = automatski tekst po kategoriji.</t>
       </text>
     </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
+    <comment ref="S1" authorId="0" shapeId="0">
       <text>
         <t>Odvojeno zarezom. Prazno = automatski popis po kategoriji.</t>
       </text>
     </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
+    <comment ref="T1" authorId="0" shapeId="0">
       <text>
         <t>JAVNO — prikazuje se kao ikona na profilu. Zalijepi @handle, instagram.com/handle ili puni URL. Prazno = bez ikone.</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
+    <comment ref="U1" authorId="0" shapeId="0">
       <text>
         <t>JAVNO — prikazuje se kao ikona na profilu. Zalijepi facebook.com/stranica ili puni URL. Prazno = bez ikone.</t>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
+    <comment ref="V1" authorId="0" shapeId="0">
       <text>
         <t>INTERNO — ne prikazuje se na stranici</t>
       </text>
     </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
+    <comment ref="W1" authorId="0" shapeId="0">
       <text>
         <t>INTERNO — ne prikazuje se na stranici</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
+    <comment ref="X1" authorId="0" shapeId="0">
       <text>
         <t>INTERNO — ne prikazuje se na stranici</t>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
+    <comment ref="Y1" authorId="0" shapeId="0">
       <text>
         <t>Za tvoje praćenje — ne utječe na import</t>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>Interno</t>
       </text>
@@ -630,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -673,154 +678,171 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>LOKACIJA I POKRIVANJE (sjedište ≠ područje rada):</t>
+          <t>KATEGORIJE:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>• grad + koordinate = SJEDIŠTE (jedna točka → jedan pin na karti). pokriva_regije = gdje pružatelj RADI.</t>
+          <t>• kategorija = PRIMARNA (određuje sliku, budžetsku grupu, slične). dodatne_kategorije = još najviše 2, odvojene ; — pružatelj se pojavljuje u svim svojim kategorijama.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>• Nema grada? Ostavi grad i koordinate prazno — pružatelj se prikazuje u listi svoje regije, bez pina. NIKAD ne izmišljaj koordinatu.</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>• Više gradova (npr. Split, Zadar, Šibenik)? grad = glavni/prvi, ostali u pokrivanje_napomena. Jedan pružatelj = jedan pin.</t>
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>LOKACIJA I POKRIVANJE (sjedište ≠ područje rada):</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• Više regija? pokriva_regije = 'Dalmacija; Kvarner'. Cijela država? pokriva_regije = 'cijela Hrvatska'.</t>
+          <t>• grad + koordinate = SJEDIŠTE (jedna točka → jedan pin na karti). pokriva_regije = gdje pružatelj RADI.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• IZNIMKA: Restorani i sale, Konobe i prostori, Najam kuće — grad i koordinate su OBAVEZNI (lokacija im je bit ponude).</t>
+          <t>• Nema grada? Ostavi grad i koordinate prazno — pružatelj se prikazuje u listi svoje regije, bez pina. NIKAD ne izmišljaj koordinatu.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• Koordinate fotografa/bendova ne moraš tražiti ručno — dovoljan je grad, geokodiranje radi skripta (Faza 1). Vrijeme uloži u točne koordinate dvorana.</t>
+          <t>• Više gradova (npr. Split, Zadar, Šibenik)? grad = glavni/prvi, ostali u pokrivanje_napomena. Jedan pružatelj = jedan pin.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>3. Prenesene recenzije (tekstualne) upisuj u list 'Recenzije' — poveži ih točnim nazivom pružatelja.</t>
+          <t>• Više regija? pokriva_regije = 'Dalmacija; Kvarner'. Cijela država? pokriva_regije = 'cijela Hrvatska'.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>4. Kad želiš podatke na stranici, spremi ovu datoteku i pokreni:  npm run import:vendors -- putanja/do/datoteke.xlsx</t>
+          <t>• IZNIMKA: Restorani i sale, Konobe i prostori, Najam kuće — grad i koordinate su OBAVEZNI (lokacija im je bit ponude).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Skripta provjerava svaki redak (koordinate, kategorije, cijene…) i ispisuje greške s brojem retka.</t>
+          <t>• Koordinate fotografa/bendova ne moraš tražiti ručno — dovoljan je grad, geokodiranje radi skripta (Faza 1). Vrijeme uloži u točne koordinate dvorana.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>5. Ako je sve u redu, generira data/vendors.json i data/profiles.json → git commit → podaci su na stranici.</t>
+          <t>3. Prenesene recenzije (tekstualne) upisuj u list 'Recenzije' — poveži ih točnim nazivom pružatelja.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>4. Kad želiš podatke na stranici, spremi ovu datoteku i pokreni:  npm run import:vendors -- putanja/do/datoteke.xlsx</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>VAŽNO — DOZVOLE:</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Skripta provjerava svaki redak (koordinate, kategorije, cijene…) i ispisuje greške s brojem retka.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>5. Ako je sve u redu, generira data/vendors.json i data/profiles.json → git commit → podaci su na stranici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>VAŽNO — DOZVOLE:</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>• Za objavu prenesenih recenzija, fotografija i ocjena zatraži suglasnost pružatelja (to je ujedno prvi kontakt za partnerstvo).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>• Kolone web/telefon/email su samo za tvoju evidenciju — import ih NE stavlja na stranicu (Direktan kontakt: zasad ne).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>• IZNIMKA: instagram i facebook SU javni — prikazuju se kao ikone na profilu pružatelja. Zalijepi @handle ili puni URL, ostalo sredi skripta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>INTERNI STATUSI (nikad javne negativne oznake):</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>• IZNIMKA: instagram i facebook SU javni — prikazuju se kao ikone na profilu pružatelja. Zalijepi @handle ili puni URL, ostalo sredi skripta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>INTERNI STATUSI (nikad javne negativne oznake):</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>• Sumnjaš da je pružatelj neaktivan, prijavljen je problem ili podaci ne valjaju? Status = Skriveno → import ga preskače (tiho uklanjanje s platforme).</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>• Detalje sumnje zapiši u kolonu napomena. Kad provjeriš i potvrdiš da je sve u redu, vrati status i pružatelj se opet uvozi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>• Redci čiji naziv počinje s 'PRIMJER' se preskaču pri importu — slobodno ih ostavi ili obriši.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>SAVJET ZA POČETAK:</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>• Redci čiji naziv počinje s 'PRIMJER' se preskaču pri importu — slobodno ih ostavi ili obriši.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>SAVJET ZA POČETAK:</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>• Kreni s 1 regijom i 2–3 kategorije (npr. Dalmacija: Restorani i sale + Foto i Video) da provjeriš cijeli tok, pa širi.</t>
         </is>
@@ -1097,34 +1119,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y6"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="46" customWidth="1" min="17" max="17"/>
-    <col width="34" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="46" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="30" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1140,115 +1163,120 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>dodatne_kategorije</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>regija*</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>grad</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>koordinate</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>pokriva_regije</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>pokrivanje_napomena</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>nacin_cijene*</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>cijena_od*</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>cijena_do</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>ocjena</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>broj_recenzija</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>izvor_ocjene</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>provjereno</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>kalendar_uzivo</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>stil</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>o_pruzatelju</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>usluge</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>web</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>telefon</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>napomena</t>
         </is>
@@ -1265,101 +1293,102 @@
           <t>Restorani i sale</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Dalmacija</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Split</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>43.5147, 16.4102</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr"/>
       <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>po osobi (raspon)</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>65</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>4.8</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>57</v>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>Google recenzije</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>DA</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>uz more, terasa</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>Terasa uz more za do 220 gostiju, vlastita kuhinja i parking. Cijena po osobi uključuje meni od 5 slijedova.</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>Meni po osobi, Osoblje, Osnovna dekoracija, Parking</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>@villa.dalmacija</t>
         </is>
       </c>
-      <c r="T2" s="4" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>facebook.com/villadalmacija</t>
         </is>
       </c>
-      <c r="U2" s="4" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>villa-dalmacija.hr</t>
         </is>
       </c>
-      <c r="V2" s="4" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>021/555-123</t>
         </is>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>info@villa-dalmacija.hr</t>
         </is>
       </c>
-      <c r="X2" s="4" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>Dozvola dobivena</t>
         </is>
       </c>
-      <c r="Y2" s="4" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>primjer — obriši ili ostavi (preskače se)</t>
         </is>
@@ -1378,89 +1407,94 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
+          <t>Audio, foto kabine i selfie mirror</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
           <t>Dalmacija</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Split</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>43.5081, 16.4402</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Dalmacija; Kvarner</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>radi u Splitu, Zadru i Šibeniku, po dogovoru i šire</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>od (paušal)</t>
         </is>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>850</v>
       </c>
-      <c r="J3" s="4" t="n"/>
-      <c r="K3" s="4" t="n">
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n">
         <v>4.8</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Google recenzije</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>DA</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>boho, film</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>Vjenčanja fotografiramo od 2014. — reportažno, s naglaskom na svjetlo i emociju.</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr"/>
-      <c r="S3" s="4" t="inlineStr">
+      <c r="S3" s="4" t="inlineStr"/>
+      <c r="T3" s="4" t="inlineStr">
         <is>
           <t>https://instagram.com/foto.anic</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="U3" s="4" t="inlineStr"/>
+      <c r="V3" s="4" t="inlineStr">
         <is>
           <t>fotostudio-anic.hr</t>
         </is>
       </c>
-      <c r="V3" s="4" t="inlineStr"/>
       <c r="W3" s="4" t="inlineStr"/>
-      <c r="X3" s="4" t="inlineStr">
+      <c r="X3" s="4" t="inlineStr"/>
+      <c r="Y3" s="4" t="inlineStr">
         <is>
           <t>Kontaktirano</t>
         </is>
       </c>
-      <c r="Y3" s="4" t="inlineStr">
+      <c r="Z3" s="4" t="inlineStr">
         <is>
           <t>primjer — preskače se pri importu</t>
         </is>
@@ -1479,57 +1513,62 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
+          <t>DJ</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
           <t>Dalmacija</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr"/>
       <c r="F4" s="4" t="inlineStr"/>
       <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>od (paušal)</t>
         </is>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>pop, rock</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr"/>
       <c r="R4" s="4" t="inlineStr"/>
       <c r="S4" s="4" t="inlineStr"/>
       <c r="T4" s="4" t="inlineStr"/>
-      <c r="U4" s="4" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr"/>
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>bend-adria.hr</t>
         </is>
       </c>
-      <c r="V4" s="4" t="inlineStr"/>
       <c r="W4" s="4" t="inlineStr"/>
-      <c r="X4" s="4" t="inlineStr">
+      <c r="X4" s="4" t="inlineStr"/>
+      <c r="Y4" s="4" t="inlineStr">
         <is>
           <t>Istraženo</t>
         </is>
       </c>
-      <c r="Y4" s="4" t="inlineStr">
+      <c r="Z4" s="4" t="inlineStr">
         <is>
           <t>primjer — bez grada/koordinata → bez pina</t>
         </is>
@@ -1546,57 +1585,58 @@
           <t>Foto i Video</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Istra</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Pula</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>na upit</t>
         </is>
       </c>
-      <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>elegantno</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr"/>
       <c r="R5" s="4" t="inlineStr"/>
       <c r="S5" s="4" t="inlineStr"/>
       <c r="T5" s="4" t="inlineStr"/>
       <c r="U5" s="4" t="inlineStr"/>
       <c r="V5" s="4" t="inlineStr"/>
       <c r="W5" s="4" t="inlineStr"/>
-      <c r="X5" s="4" t="inlineStr">
+      <c r="X5" s="4" t="inlineStr"/>
+      <c r="Y5" s="4" t="inlineStr">
         <is>
           <t>Istraženo</t>
         </is>
       </c>
-      <c r="Y5" s="4" t="inlineStr">
+      <c r="Z5" s="4" t="inlineStr">
         <is>
           <t>primjer — koordinate se geokodiraju iz grada</t>
         </is>
@@ -1613,93 +1653,94 @@
           <t>Organizatori vjenčanja</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Zagreb i okolica</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Zagreb</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>45.8150, 15.9819</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>cijela Hrvatska</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>organiziramo vjenčanja u cijeloj Hrvatskoj</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>na upit</t>
         </is>
       </c>
-      <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
-      <c r="K6" s="4" t="n">
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Google recenzije</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>DA</t>
         </is>
       </c>
-      <c r="O6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>full service</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t>Organiziramo vjenčanja od Istre do Slavonije — od koncepta do izvedbe.</t>
         </is>
       </c>
-      <c r="R6" s="4" t="inlineStr"/>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="S6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>@perfectday.hr</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
+      <c r="U6" s="4" t="inlineStr">
         <is>
           <t>facebook.com/perfectdayweddings</t>
         </is>
       </c>
-      <c r="U6" s="4" t="inlineStr">
+      <c r="V6" s="4" t="inlineStr">
         <is>
           <t>perfectday.hr</t>
         </is>
       </c>
-      <c r="V6" s="4" t="inlineStr"/>
       <c r="W6" s="4" t="inlineStr"/>
-      <c r="X6" s="4" t="inlineStr">
+      <c r="X6" s="4" t="inlineStr"/>
+      <c r="Y6" s="4" t="inlineStr">
         <is>
           <t>Dozvola dobivena</t>
         </is>
       </c>
-      <c r="Y6" s="4" t="inlineStr">
+      <c r="Z6" s="4" t="inlineStr">
         <is>
           <t>primjer — pokriva cijelu HR</t>
         </is>
@@ -1710,19 +1751,19 @@
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Sifrarnici!$A$1:$A$28</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Sifrarnici!$B$1:$B$5</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"od (paušal),po osobi (raspon)"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"DA,NE"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"DA,NE"</formula1>
     </dataValidation>
-    <dataValidation sqref="X2:X500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"DA,NE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y2:Y500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Sifrarnici!$C$1:$C$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>